<commit_message>
Upgrade SNOW dossier for analyst recruiting
</commit_message>
<xml_diff>
--- a/model/Model.xlsx
+++ b/model/Model.xlsx
@@ -156,27 +156,27 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A1:N1" displayName="Table_1" name="Table_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://customooxmlschemas.google.com/" headerRowCount="1" ref="A1:N13" displayName="Table_1" name="Table_1" id="1">
   <tableColumns count="14">
-    <tableColumn name="Column1" id="1"/>
-    <tableColumn name="Column2" id="2"/>
-    <tableColumn name="Column3" id="3"/>
-    <tableColumn name="Column4" id="4"/>
-    <tableColumn name="Column5" id="5"/>
-    <tableColumn name="Column6" id="6"/>
-    <tableColumn name="Column7" id="7"/>
-    <tableColumn name="Column8" id="8"/>
-    <tableColumn name="Column9" id="9"/>
-    <tableColumn name="Column10" id="10"/>
-    <tableColumn name="Column11" id="11"/>
-    <tableColumn name="Column12" id="12"/>
-    <tableColumn name="Column13" id="13"/>
-    <tableColumn name="Column14" id="14"/>
+    <tableColumn name="quarter" id="1"/>
+    <tableColumn name="revenue" id="2"/>
+    <tableColumn name="yoy_growth_%" id="3"/>
+    <tableColumn name="gross_margin_%" id="4"/>
+    <tableColumn name="s&amp;m_%rev" id="5"/>
+    <tableColumn name="r&amp;d_%rev" id="6"/>
+    <tableColumn name="g&amp;a_%rev" id="7"/>
+    <tableColumn name="arr" id="8"/>
+    <tableColumn name="nrr_%" id="9"/>
+    <tableColumn name="churn_%" id="10"/>
+    <tableColumn name="arpu" id="11"/>
+    <tableColumn name="cfo" id="12"/>
+    <tableColumn name="capex" id="13"/>
+    <tableColumn name="fcf" id="14"/>
   </tableColumns>
   <tableStyleInfo name="KPI_History-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion1">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" headerRowCount="1"/>
+      <ns1:sheetsCustomData headerRowCount="1"/>
     </ext>
   </extLst>
 </table>
@@ -377,7 +377,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -439,6 +439,558 @@
       <c r="Y1" s="3"/>
       <c r="Z1" s="3"/>
     </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>FY24-Q1</t>
+        </is>
+      </c>
+      <c r="B2" s="0">
+        <v>624</v>
+      </c>
+      <c r="C2" s="0">
+        <v>48.0</v>
+      </c>
+      <c r="D2" s="0">
+        <v>76.5</v>
+      </c>
+      <c r="E2" s="0">
+        <v>48.0</v>
+      </c>
+      <c r="F2" s="0">
+        <v>24.0</v>
+      </c>
+      <c r="G2" s="0">
+        <v>11.5</v>
+      </c>
+      <c r="H2" s="0">
+        <v>2810</v>
+      </c>
+      <c r="I2" s="0">
+        <v>131</v>
+      </c>
+      <c r="J2" s="0">
+        <v>7.5</v>
+      </c>
+      <c r="K2" s="0">
+        <v>196000</v>
+      </c>
+      <c r="L2" s="0">
+        <v>168</v>
+      </c>
+      <c r="M2" s="0">
+        <v>24</v>
+      </c>
+      <c r="N2" s="0">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>FY24-Q2</t>
+        </is>
+      </c>
+      <c r="B3" s="0">
+        <v>674</v>
+      </c>
+      <c r="C3" s="0">
+        <v>37.5</v>
+      </c>
+      <c r="D3" s="0">
+        <v>76.0</v>
+      </c>
+      <c r="E3" s="0">
+        <v>47.0</v>
+      </c>
+      <c r="F3" s="0">
+        <v>24.5</v>
+      </c>
+      <c r="G3" s="0">
+        <v>11.0</v>
+      </c>
+      <c r="H3" s="0">
+        <v>2950</v>
+      </c>
+      <c r="I3" s="0">
+        <v>128</v>
+      </c>
+      <c r="J3" s="0">
+        <v>8.0</v>
+      </c>
+      <c r="K3" s="0">
+        <v>201000</v>
+      </c>
+      <c r="L3" s="0">
+        <v>176</v>
+      </c>
+      <c r="M3" s="0">
+        <v>26</v>
+      </c>
+      <c r="N3" s="0">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>FY24-Q3</t>
+        </is>
+      </c>
+      <c r="B4" s="0">
+        <v>734</v>
+      </c>
+      <c r="C4" s="0">
+        <v>32.0</v>
+      </c>
+      <c r="D4" s="0">
+        <v>75.5</v>
+      </c>
+      <c r="E4" s="0">
+        <v>46.0</v>
+      </c>
+      <c r="F4" s="0">
+        <v>24.5</v>
+      </c>
+      <c r="G4" s="0">
+        <v>10.8</v>
+      </c>
+      <c r="H4" s="0">
+        <v>3120</v>
+      </c>
+      <c r="I4" s="0">
+        <v>126</v>
+      </c>
+      <c r="J4" s="0">
+        <v>8.5</v>
+      </c>
+      <c r="K4" s="0">
+        <v>207000</v>
+      </c>
+      <c r="L4" s="0">
+        <v>190</v>
+      </c>
+      <c r="M4" s="0">
+        <v>28</v>
+      </c>
+      <c r="N4" s="0">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>FY24-Q4</t>
+        </is>
+      </c>
+      <c r="B5" s="0">
+        <v>775</v>
+      </c>
+      <c r="C5" s="0">
+        <v>30.0</v>
+      </c>
+      <c r="D5" s="0">
+        <v>75.0</v>
+      </c>
+      <c r="E5" s="0">
+        <v>45.0</v>
+      </c>
+      <c r="F5" s="0">
+        <v>24.0</v>
+      </c>
+      <c r="G5" s="0">
+        <v>10.5</v>
+      </c>
+      <c r="H5" s="0">
+        <v>3280</v>
+      </c>
+      <c r="I5" s="0">
+        <v>124</v>
+      </c>
+      <c r="J5" s="0">
+        <v>9.0</v>
+      </c>
+      <c r="K5" s="0">
+        <v>214000</v>
+      </c>
+      <c r="L5" s="0">
+        <v>205</v>
+      </c>
+      <c r="M5" s="0">
+        <v>30</v>
+      </c>
+      <c r="N5" s="0">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>FY25-Q1</t>
+        </is>
+      </c>
+      <c r="B6" s="0">
+        <v>828</v>
+      </c>
+      <c r="C6" s="0">
+        <v>32.7</v>
+      </c>
+      <c r="D6" s="0">
+        <v>75.3</v>
+      </c>
+      <c r="E6" s="0">
+        <v>44.5</v>
+      </c>
+      <c r="F6" s="0">
+        <v>23.8</v>
+      </c>
+      <c r="G6" s="0">
+        <v>10.4</v>
+      </c>
+      <c r="H6" s="0">
+        <v>3450</v>
+      </c>
+      <c r="I6" s="0">
+        <v>123</v>
+      </c>
+      <c r="J6" s="0">
+        <v>9.0</v>
+      </c>
+      <c r="K6" s="0">
+        <v>223000</v>
+      </c>
+      <c r="L6" s="0">
+        <v>222</v>
+      </c>
+      <c r="M6" s="0">
+        <v>32</v>
+      </c>
+      <c r="N6" s="0">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>FY25-Q2</t>
+        </is>
+      </c>
+      <c r="B7" s="0">
+        <v>874</v>
+      </c>
+      <c r="C7" s="0">
+        <v>29.7</v>
+      </c>
+      <c r="D7" s="0">
+        <v>75.1</v>
+      </c>
+      <c r="E7" s="0">
+        <v>44.0</v>
+      </c>
+      <c r="F7" s="0">
+        <v>23.5</v>
+      </c>
+      <c r="G7" s="0">
+        <v>10.2</v>
+      </c>
+      <c r="H7" s="0">
+        <v>3600</v>
+      </c>
+      <c r="I7" s="0">
+        <v>122</v>
+      </c>
+      <c r="J7" s="0">
+        <v>9.2</v>
+      </c>
+      <c r="K7" s="0">
+        <v>230000</v>
+      </c>
+      <c r="L7" s="0">
+        <v>236</v>
+      </c>
+      <c r="M7" s="0">
+        <v>34</v>
+      </c>
+      <c r="N7" s="0">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>FY25-Q3</t>
+        </is>
+      </c>
+      <c r="B8" s="0">
+        <v>920</v>
+      </c>
+      <c r="C8" s="0">
+        <v>25.3</v>
+      </c>
+      <c r="D8" s="0">
+        <v>74.9</v>
+      </c>
+      <c r="E8" s="0">
+        <v>43.8</v>
+      </c>
+      <c r="F8" s="0">
+        <v>23.3</v>
+      </c>
+      <c r="G8" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="H8" s="0">
+        <v>3770</v>
+      </c>
+      <c r="I8" s="0">
+        <v>121</v>
+      </c>
+      <c r="J8" s="0">
+        <v>9.3</v>
+      </c>
+      <c r="K8" s="0">
+        <v>238000</v>
+      </c>
+      <c r="L8" s="0">
+        <v>249</v>
+      </c>
+      <c r="M8" s="0">
+        <v>35</v>
+      </c>
+      <c r="N8" s="0">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>FY25-Q4</t>
+        </is>
+      </c>
+      <c r="B9" s="0">
+        <v>964</v>
+      </c>
+      <c r="C9" s="0">
+        <v>24.4</v>
+      </c>
+      <c r="D9" s="0">
+        <v>74.8</v>
+      </c>
+      <c r="E9" s="0">
+        <v>43.5</v>
+      </c>
+      <c r="F9" s="0">
+        <v>23.0</v>
+      </c>
+      <c r="G9" s="0">
+        <v>9.8</v>
+      </c>
+      <c r="H9" s="0">
+        <v>3940</v>
+      </c>
+      <c r="I9" s="0">
+        <v>120</v>
+      </c>
+      <c r="J9" s="0">
+        <v>9.5</v>
+      </c>
+      <c r="K9" s="0">
+        <v>246000</v>
+      </c>
+      <c r="L9" s="0">
+        <v>262</v>
+      </c>
+      <c r="M9" s="0">
+        <v>36</v>
+      </c>
+      <c r="N9" s="0">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>FY26E-Q1</t>
+        </is>
+      </c>
+      <c r="B10" s="0">
+        <v>1010</v>
+      </c>
+      <c r="C10" s="0">
+        <v>22.0</v>
+      </c>
+      <c r="D10" s="0">
+        <v>74.5</v>
+      </c>
+      <c r="E10" s="0">
+        <v>43.0</v>
+      </c>
+      <c r="F10" s="0">
+        <v>22.8</v>
+      </c>
+      <c r="G10" s="0">
+        <v>9.7</v>
+      </c>
+      <c r="H10" s="0">
+        <v>4120</v>
+      </c>
+      <c r="I10" s="0">
+        <v>118</v>
+      </c>
+      <c r="J10" s="0">
+        <v>9.8</v>
+      </c>
+      <c r="K10" s="0">
+        <v>254000</v>
+      </c>
+      <c r="L10" s="0">
+        <v>278</v>
+      </c>
+      <c r="M10" s="0">
+        <v>38</v>
+      </c>
+      <c r="N10" s="0">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>FY26E-Q2</t>
+        </is>
+      </c>
+      <c r="B11" s="0">
+        <v>1060</v>
+      </c>
+      <c r="C11" s="0">
+        <v>21.3</v>
+      </c>
+      <c r="D11" s="0">
+        <v>74.3</v>
+      </c>
+      <c r="E11" s="0">
+        <v>42.7</v>
+      </c>
+      <c r="F11" s="0">
+        <v>22.5</v>
+      </c>
+      <c r="G11" s="0">
+        <v>9.5</v>
+      </c>
+      <c r="H11" s="0">
+        <v>4300</v>
+      </c>
+      <c r="I11" s="0">
+        <v>117</v>
+      </c>
+      <c r="J11" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="K11" s="0">
+        <v>262000</v>
+      </c>
+      <c r="L11" s="0">
+        <v>293</v>
+      </c>
+      <c r="M11" s="0">
+        <v>39</v>
+      </c>
+      <c r="N11" s="0">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>FY26E-Q3</t>
+        </is>
+      </c>
+      <c r="B12" s="0">
+        <v>1115</v>
+      </c>
+      <c r="C12" s="0">
+        <v>21.2</v>
+      </c>
+      <c r="D12" s="0">
+        <v>74.1</v>
+      </c>
+      <c r="E12" s="0">
+        <v>42.4</v>
+      </c>
+      <c r="F12" s="0">
+        <v>22.3</v>
+      </c>
+      <c r="G12" s="0">
+        <v>9.4</v>
+      </c>
+      <c r="H12" s="0">
+        <v>4490</v>
+      </c>
+      <c r="I12" s="0">
+        <v>116</v>
+      </c>
+      <c r="J12" s="0">
+        <v>10.2</v>
+      </c>
+      <c r="K12" s="0">
+        <v>271000</v>
+      </c>
+      <c r="L12" s="0">
+        <v>308</v>
+      </c>
+      <c r="M12" s="0">
+        <v>40</v>
+      </c>
+      <c r="N12" s="0">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>FY26E-Q4</t>
+        </is>
+      </c>
+      <c r="B13" s="0">
+        <v>1170</v>
+      </c>
+      <c r="C13" s="0">
+        <v>21.4</v>
+      </c>
+      <c r="D13" s="0">
+        <v>74.0</v>
+      </c>
+      <c r="E13" s="0">
+        <v>42.0</v>
+      </c>
+      <c r="F13" s="0">
+        <v>22.0</v>
+      </c>
+      <c r="G13" s="0">
+        <v>9.2</v>
+      </c>
+      <c r="H13" s="0">
+        <v>4685</v>
+      </c>
+      <c r="I13" s="0">
+        <v>115</v>
+      </c>
+      <c r="J13" s="0">
+        <v>10.5</v>
+      </c>
+      <c r="K13" s="0">
+        <v>280000</v>
+      </c>
+      <c r="L13" s="0">
+        <v>324</v>
+      </c>
+      <c r="M13" s="0">
+        <v>42</v>
+      </c>
+      <c r="N13" s="0">
+        <v>282</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
   <tableParts count="1">

</xml_diff>